<commit_message>
implemented all four types of rate control, not fully tested yet
</commit_message>
<xml_diff>
--- a/aln_control/testCases.xlsx
+++ b/aln_control/testCases.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Promotion\neurolib\aln_control\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDCFBEB1-8673-43DA-931A-908A928B848F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE2DE18-4A97-4965-A1F4-96147AF23582}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-3120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-3120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Tabelle2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="45">
   <si>
     <t>TC</t>
   </si>
@@ -132,13 +133,49 @@
   </si>
   <si>
     <t>different solutions for different initial guess, non-vanishing gradient</t>
+  </si>
+  <si>
+    <t>start</t>
+  </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
+    <t>high</t>
+  </si>
+  <si>
+    <t>fast</t>
+  </si>
+  <si>
+    <t>slow</t>
+  </si>
+  <si>
+    <t>B.3.a: at low state, rate derivative wrt mu is zero, so no change in possible</t>
+  </si>
+  <si>
+    <t>2,3,4,5</t>
+  </si>
+  <si>
+    <t>initial a</t>
+  </si>
+  <si>
+    <t>initial b</t>
+  </si>
+  <si>
+    <t>random</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>zero</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -177,6 +214,19 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -568,7 +618,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -683,8 +733,32 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Gut" xfId="1" builtinId="26"/>
@@ -968,164 +1042,167 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB52"/>
+  <dimension ref="A1:AE53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="12" width="9.85546875" customWidth="1"/>
-    <col min="14" max="28" width="9.85546875" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" customWidth="1"/>
+    <col min="6" max="6" width="4" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="3.7109375" customWidth="1"/>
+    <col min="9" max="15" width="6.42578125" customWidth="1"/>
+    <col min="16" max="16" width="3" customWidth="1"/>
+    <col min="17" max="23" width="6.42578125" customWidth="1"/>
+    <col min="24" max="24" width="3" customWidth="1"/>
+    <col min="25" max="31" width="6.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="D1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="1">
-        <v>0</v>
-      </c>
-      <c r="G1" s="1">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="1">
+      <c r="G1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" s="1">
+        <v>0</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2</v>
+      </c>
+      <c r="K1" s="1">
         <v>4</v>
       </c>
-      <c r="I1" s="1">
+      <c r="L1" s="1">
         <v>6</v>
       </c>
-      <c r="J1" s="1">
+      <c r="M1" s="1">
         <v>8</v>
       </c>
-      <c r="K1" s="1">
+      <c r="N1" s="1">
         <v>10</v>
       </c>
-      <c r="L1" s="1">
+      <c r="O1" s="1">
         <v>12</v>
       </c>
-      <c r="N1" s="1">
+      <c r="Q1" s="1">
         <v>1</v>
       </c>
-      <c r="O1" s="1">
+      <c r="R1" s="1">
         <v>3</v>
       </c>
-      <c r="P1" s="1">
+      <c r="S1" s="1">
         <v>5</v>
       </c>
-      <c r="Q1" s="1">
+      <c r="T1" s="1">
         <v>7</v>
       </c>
-      <c r="R1" s="1">
+      <c r="U1" s="1">
         <v>9</v>
       </c>
-      <c r="S1" s="1">
+      <c r="V1" s="1">
         <v>11</v>
       </c>
-      <c r="T1" s="1">
+      <c r="W1" s="1">
         <v>13</v>
       </c>
-      <c r="U1"/>
-      <c r="V1" s="1">
+      <c r="X1"/>
+      <c r="Y1" s="1">
         <v>14</v>
       </c>
-      <c r="W1" s="1">
+      <c r="Z1" s="1">
         <v>15</v>
       </c>
-      <c r="X1" s="1">
+      <c r="AA1" s="1">
         <v>16</v>
       </c>
-      <c r="Y1" s="1">
+      <c r="AB1" s="1">
         <v>17</v>
       </c>
-      <c r="Z1" s="1">
+      <c r="AC1" s="1">
         <v>18</v>
       </c>
-      <c r="AA1" s="1">
+      <c r="AD1" s="1">
         <v>19</v>
       </c>
-      <c r="AB1" s="1">
+      <c r="AE1" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="D3" t="s">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
         <v>1</v>
       </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
         <v>2</v>
       </c>
-      <c r="H3">
+      <c r="K3">
         <v>1</v>
       </c>
-      <c r="I3">
+      <c r="L3">
         <v>0.1</v>
       </c>
-      <c r="J3">
+      <c r="M3">
         <v>0.2</v>
       </c>
-      <c r="K3">
+      <c r="N3">
         <v>1.2</v>
       </c>
-      <c r="L3" t="s">
+      <c r="O3" t="s">
         <v>17</v>
       </c>
-      <c r="N3">
+      <c r="Q3">
         <v>1</v>
       </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
         <v>2</v>
       </c>
-      <c r="Q3">
+      <c r="T3">
         <v>0.1</v>
       </c>
-      <c r="R3">
+      <c r="U3">
         <v>0.2</v>
       </c>
-      <c r="S3">
+      <c r="V3">
         <v>1.2</v>
       </c>
-      <c r="T3" t="s">
+      <c r="W3" t="s">
         <v>17</v>
       </c>
-      <c r="V3">
-        <v>0</v>
-      </c>
-      <c r="W3">
+      <c r="Y3">
+        <v>0</v>
+      </c>
+      <c r="Z3">
         <v>1</v>
       </c>
-      <c r="X3">
+      <c r="AA3">
         <v>2</v>
       </c>
-      <c r="Y3">
+      <c r="AB3">
         <v>0.1</v>
       </c>
-      <c r="Z3">
+      <c r="AC3">
         <v>0.2</v>
       </c>
-      <c r="AA3">
+      <c r="AD3">
         <v>1.2</v>
       </c>
-      <c r="AB3" t="s">
+      <c r="AE3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
         <v>2</v>
       </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
       <c r="I4">
         <v>0</v>
       </c>
@@ -1138,14 +1215,14 @@
       <c r="L4">
         <v>0</v>
       </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
       <c r="N4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O4">
-        <v>1</v>
-      </c>
-      <c r="P4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>1</v>
@@ -1159,14 +1236,14 @@
       <c r="T4">
         <v>1</v>
       </c>
+      <c r="U4">
+        <v>1</v>
+      </c>
       <c r="V4">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="W4">
-        <v>0.1</v>
-      </c>
-      <c r="X4">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="Y4">
         <v>0.1</v>
@@ -1180,760 +1257,870 @@
       <c r="AB4">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="5" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC4">
+        <v>0.1</v>
+      </c>
+      <c r="AD4">
+        <v>0.1</v>
+      </c>
+      <c r="AE4">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="35"/>
-      <c r="G6" s="36"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="36"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="36"/>
-      <c r="L6" s="39"/>
-      <c r="N6" s="55"/>
-      <c r="O6" s="56"/>
-      <c r="P6" s="57"/>
-      <c r="Q6" s="57"/>
+      <c r="C6" s="1"/>
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6" s="35"/>
+      <c r="J6" s="36"/>
+      <c r="K6" s="37"/>
+      <c r="L6" s="36"/>
+      <c r="M6" s="38"/>
+      <c r="N6" s="36"/>
+      <c r="O6" s="39"/>
+      <c r="Q6" s="55"/>
       <c r="R6" s="56"/>
-      <c r="S6" s="56"/>
-      <c r="T6" s="58"/>
-      <c r="V6" s="35"/>
-      <c r="W6" s="56"/>
-      <c r="X6" s="38"/>
-      <c r="Y6" s="56"/>
-      <c r="Z6" s="38"/>
-      <c r="AA6" s="56"/>
-      <c r="AB6" s="39"/>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="S6" s="57"/>
+      <c r="T6" s="57"/>
+      <c r="U6" s="56"/>
+      <c r="V6" s="56"/>
+      <c r="W6" s="58"/>
+      <c r="Y6" s="35"/>
+      <c r="Z6" s="56"/>
+      <c r="AA6" s="38"/>
+      <c r="AB6" s="56"/>
+      <c r="AC6" s="38"/>
+      <c r="AD6" s="56"/>
+      <c r="AE6" s="39"/>
+    </row>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="40"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
-      <c r="I7" s="41"/>
-      <c r="J7" s="42"/>
-      <c r="K7" s="41"/>
-      <c r="L7" s="43"/>
-      <c r="N7" s="59"/>
-      <c r="O7" s="41"/>
-      <c r="P7" s="60"/>
-      <c r="Q7" s="60"/>
+      <c r="C7" s="1"/>
+      <c r="I7" s="40"/>
+      <c r="J7" s="41"/>
+      <c r="K7" s="42"/>
+      <c r="L7" s="41"/>
+      <c r="M7" s="42"/>
+      <c r="N7" s="41"/>
+      <c r="O7" s="43"/>
+      <c r="Q7" s="59"/>
       <c r="R7" s="41"/>
-      <c r="S7" s="41"/>
-      <c r="T7" s="61"/>
-      <c r="V7" s="40"/>
-      <c r="W7" s="41"/>
-      <c r="X7" s="42"/>
-      <c r="Y7" s="41"/>
-      <c r="Z7" s="3"/>
-      <c r="AA7" s="41"/>
-      <c r="AB7" s="43"/>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="S7" s="60"/>
+      <c r="T7" s="60"/>
+      <c r="U7" s="41"/>
+      <c r="V7" s="41"/>
+      <c r="W7" s="61"/>
+      <c r="Y7" s="40"/>
+      <c r="Z7" s="41"/>
+      <c r="AA7" s="42"/>
+      <c r="AB7" s="41"/>
+      <c r="AC7" s="3"/>
+      <c r="AD7" s="41"/>
+      <c r="AE7" s="43"/>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="44"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
-      <c r="I8" s="45"/>
-      <c r="J8" s="46"/>
-      <c r="K8" s="45"/>
-      <c r="L8" s="47"/>
-      <c r="N8" s="85"/>
-      <c r="O8" s="87"/>
-      <c r="P8" s="73"/>
-      <c r="Q8" s="93"/>
-      <c r="R8" s="5"/>
-      <c r="S8" s="77"/>
-      <c r="T8" s="21"/>
-      <c r="V8" s="89"/>
-      <c r="W8" s="5"/>
-      <c r="X8" s="2"/>
-      <c r="Y8" s="5"/>
-      <c r="Z8" s="92"/>
-      <c r="AA8" s="5"/>
-      <c r="AB8" s="18"/>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C8" s="1"/>
+      <c r="D8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="I8" s="44"/>
+      <c r="J8" s="45"/>
+      <c r="K8" s="46"/>
+      <c r="L8" s="45"/>
+      <c r="M8" s="46"/>
+      <c r="N8" s="45"/>
+      <c r="O8" s="47"/>
+      <c r="Q8" s="85"/>
+      <c r="R8" s="87"/>
+      <c r="S8" s="73"/>
+      <c r="T8" s="93"/>
+      <c r="U8" s="5"/>
+      <c r="V8" s="77"/>
+      <c r="W8" s="21"/>
+      <c r="Y8" s="89"/>
+      <c r="Z8" s="5"/>
+      <c r="AA8" s="2"/>
+      <c r="AB8" s="5"/>
+      <c r="AC8" s="92"/>
+      <c r="AD8" s="5"/>
+      <c r="AE8" s="18"/>
+    </row>
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="48"/>
-      <c r="H9" s="49"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="48"/>
-      <c r="L9" s="15"/>
-      <c r="N9" s="86"/>
-      <c r="O9" s="88"/>
-      <c r="P9" s="74"/>
-      <c r="Q9" s="107"/>
-      <c r="R9" s="7"/>
-      <c r="S9" s="78"/>
-      <c r="T9" s="22"/>
-      <c r="V9" s="108"/>
-      <c r="W9" s="7"/>
-      <c r="X9" s="4"/>
-      <c r="Y9" s="7"/>
-      <c r="Z9" s="114"/>
-      <c r="AA9" s="7"/>
-      <c r="AB9" s="15"/>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C9" s="1"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="48"/>
+      <c r="K9" s="49"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="48"/>
+      <c r="O9" s="15"/>
+      <c r="Q9" s="86"/>
+      <c r="R9" s="88"/>
+      <c r="S9" s="74"/>
+      <c r="T9" s="107"/>
+      <c r="U9" s="7"/>
+      <c r="V9" s="78"/>
+      <c r="W9" s="22"/>
+      <c r="Y9" s="108"/>
+      <c r="Z9" s="7"/>
+      <c r="AA9" s="4"/>
+      <c r="AB9" s="7"/>
+      <c r="AC9" s="110"/>
+      <c r="AD9" s="7"/>
+      <c r="AE9" s="15"/>
+    </row>
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="H10" s="42"/>
-      <c r="I10" s="41"/>
-      <c r="J10" s="42"/>
-      <c r="K10" s="41"/>
-      <c r="L10" s="43"/>
-      <c r="N10" s="44"/>
-      <c r="O10" s="5"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="5"/>
-      <c r="R10" s="113"/>
-      <c r="S10" s="5"/>
-      <c r="T10" s="18"/>
-      <c r="V10" s="16"/>
-      <c r="W10" s="41"/>
-      <c r="X10" s="3"/>
-      <c r="Y10" s="6"/>
-      <c r="Z10" s="3"/>
-      <c r="AA10" s="41"/>
-      <c r="AB10" s="19"/>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C10" s="1"/>
+      <c r="D10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10" s="40"/>
+      <c r="J10" s="41"/>
+      <c r="K10" s="42"/>
+      <c r="L10" s="41"/>
+      <c r="M10" s="42"/>
+      <c r="N10" s="41"/>
+      <c r="O10" s="43"/>
+      <c r="Q10" s="44"/>
+      <c r="R10" s="5"/>
+      <c r="S10" s="2"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="113"/>
+      <c r="V10" s="5"/>
+      <c r="W10" s="18"/>
+      <c r="Y10" s="16"/>
+      <c r="Z10" s="41"/>
+      <c r="AA10" s="3"/>
+      <c r="AB10" s="6"/>
+      <c r="AC10" s="3"/>
+      <c r="AD10" s="41"/>
+      <c r="AE10" s="19"/>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="40"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="43"/>
-      <c r="N11" s="91"/>
-      <c r="O11" s="7"/>
-      <c r="P11" s="4"/>
-      <c r="Q11" s="7"/>
-      <c r="R11" s="114"/>
-      <c r="S11" s="7"/>
-      <c r="T11" s="15"/>
-      <c r="V11" s="16"/>
-      <c r="W11" s="41"/>
-      <c r="X11" s="3"/>
-      <c r="Y11" s="6"/>
-      <c r="Z11" s="3"/>
-      <c r="AA11" s="41"/>
-      <c r="AB11" s="19"/>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C11" s="1"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="43"/>
+      <c r="Q11" s="91"/>
+      <c r="R11" s="7"/>
+      <c r="S11" s="4"/>
+      <c r="T11" s="7"/>
+      <c r="U11" s="115"/>
+      <c r="V11" s="7"/>
+      <c r="W11" s="15"/>
+      <c r="Y11" s="16"/>
+      <c r="Z11" s="41"/>
+      <c r="AA11" s="3"/>
+      <c r="AB11" s="6"/>
+      <c r="AC11" s="3"/>
+      <c r="AD11" s="41"/>
+      <c r="AE11" s="19"/>
+    </row>
+    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="44"/>
-      <c r="G12" s="45"/>
-      <c r="H12" s="46"/>
-      <c r="I12" s="45"/>
-      <c r="J12" s="46"/>
-      <c r="K12" s="45"/>
-      <c r="L12" s="47"/>
-      <c r="N12" s="16"/>
-      <c r="O12" s="104"/>
-      <c r="P12" s="3"/>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="3"/>
-      <c r="S12" s="104"/>
-      <c r="T12" s="19"/>
-      <c r="V12" s="17"/>
-      <c r="W12" s="5"/>
-      <c r="X12" s="109"/>
-      <c r="Y12" s="5"/>
-      <c r="Z12" s="2"/>
-      <c r="AA12" s="5"/>
-      <c r="AB12" s="67"/>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C12" s="1"/>
+      <c r="D12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" t="s">
+        <v>34</v>
+      </c>
+      <c r="I12" s="44"/>
+      <c r="J12" s="45"/>
+      <c r="K12" s="46"/>
+      <c r="L12" s="45"/>
+      <c r="M12" s="46"/>
+      <c r="N12" s="45"/>
+      <c r="O12" s="47"/>
+      <c r="Q12" s="16"/>
+      <c r="R12" s="104"/>
+      <c r="S12" s="3"/>
+      <c r="T12" s="6"/>
+      <c r="U12" s="3"/>
+      <c r="V12" s="104"/>
+      <c r="W12" s="19"/>
+      <c r="Y12" s="17"/>
+      <c r="Z12" s="5"/>
+      <c r="AA12" s="109"/>
+      <c r="AB12" s="5"/>
+      <c r="AC12" s="2"/>
+      <c r="AD12" s="5"/>
+      <c r="AE12" s="67"/>
+    </row>
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F13" s="50"/>
-      <c r="G13" s="48"/>
-      <c r="H13" s="49"/>
-      <c r="I13" s="48"/>
-      <c r="J13" s="49"/>
-      <c r="K13" s="48"/>
-      <c r="L13" s="54"/>
-      <c r="N13" s="16"/>
-      <c r="O13" s="104"/>
-      <c r="P13" s="3"/>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="3"/>
-      <c r="S13" s="104"/>
-      <c r="T13" s="19"/>
-      <c r="V13" s="14"/>
-      <c r="W13" s="7"/>
-      <c r="X13" s="110"/>
-      <c r="Y13" s="7"/>
-      <c r="Z13" s="4"/>
-      <c r="AA13" s="7"/>
-      <c r="AB13" s="111"/>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C13" s="1"/>
+      <c r="I13" s="50"/>
+      <c r="J13" s="48"/>
+      <c r="K13" s="49"/>
+      <c r="L13" s="48"/>
+      <c r="M13" s="49"/>
+      <c r="N13" s="48"/>
+      <c r="O13" s="54"/>
+      <c r="Q13" s="16"/>
+      <c r="R13" s="104"/>
+      <c r="S13" s="3"/>
+      <c r="T13" s="6"/>
+      <c r="U13" s="3"/>
+      <c r="V13" s="104"/>
+      <c r="W13" s="19"/>
+      <c r="Y13" s="14"/>
+      <c r="Z13" s="7"/>
+      <c r="AA13" s="110"/>
+      <c r="AB13" s="7"/>
+      <c r="AC13" s="4"/>
+      <c r="AD13" s="7"/>
+      <c r="AE13" s="111"/>
+    </row>
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F14" s="40"/>
-      <c r="G14" s="41"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="41"/>
-      <c r="J14" s="42"/>
-      <c r="K14" s="41"/>
-      <c r="L14" s="43"/>
-      <c r="N14" s="17"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="75"/>
-      <c r="Q14" s="5"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="5"/>
-      <c r="T14" s="67"/>
-      <c r="V14" s="16"/>
-      <c r="W14" s="6"/>
-      <c r="X14" s="3"/>
-      <c r="Y14" s="34"/>
-      <c r="Z14" s="3"/>
-      <c r="AA14" s="6"/>
-      <c r="AB14" s="19"/>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C14" s="1"/>
+      <c r="D14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" t="s">
+        <v>36</v>
+      </c>
+      <c r="I14" s="40"/>
+      <c r="J14" s="41"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="41"/>
+      <c r="M14" s="42"/>
+      <c r="N14" s="41"/>
+      <c r="O14" s="43"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="5"/>
+      <c r="S14" s="75"/>
+      <c r="T14" s="5"/>
+      <c r="U14" s="2"/>
+      <c r="V14" s="5"/>
+      <c r="W14" s="67"/>
+      <c r="Y14" s="16"/>
+      <c r="Z14" s="6"/>
+      <c r="AA14" s="3"/>
+      <c r="AB14" s="34"/>
+      <c r="AC14" s="3"/>
+      <c r="AD14" s="6"/>
+      <c r="AE14" s="19"/>
+    </row>
+    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F15" s="40"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="42"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="43"/>
-      <c r="N15" s="14"/>
-      <c r="O15" s="7"/>
-      <c r="P15" s="76"/>
-      <c r="Q15" s="7"/>
-      <c r="R15" s="4"/>
-      <c r="S15" s="7"/>
-      <c r="T15" s="90"/>
-      <c r="V15" s="16"/>
-      <c r="W15" s="6"/>
-      <c r="X15" s="3"/>
-      <c r="Y15" s="64"/>
-      <c r="Z15" s="3"/>
-      <c r="AA15" s="6"/>
-      <c r="AB15" s="19"/>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C15" s="1"/>
+      <c r="I15" s="40"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="42"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="43"/>
+      <c r="Q15" s="14"/>
+      <c r="R15" s="7"/>
+      <c r="S15" s="76"/>
+      <c r="T15" s="7"/>
+      <c r="U15" s="4"/>
+      <c r="V15" s="7"/>
+      <c r="W15" s="90"/>
+      <c r="Y15" s="16"/>
+      <c r="Z15" s="6"/>
+      <c r="AA15" s="3"/>
+      <c r="AB15" s="64"/>
+      <c r="AC15" s="3"/>
+      <c r="AD15" s="6"/>
+      <c r="AE15" s="19"/>
+    </row>
+    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F16" s="44"/>
-      <c r="G16" s="45"/>
-      <c r="H16" s="46"/>
-      <c r="I16" s="45"/>
-      <c r="J16" s="46"/>
-      <c r="K16" s="45"/>
-      <c r="L16" s="47"/>
-      <c r="N16" s="16"/>
-      <c r="O16" s="6"/>
-      <c r="P16" s="3"/>
-      <c r="Q16" s="41"/>
-      <c r="R16" s="3"/>
-      <c r="S16" s="6"/>
-      <c r="T16" s="19"/>
-      <c r="V16" s="105"/>
-      <c r="W16" s="5"/>
-      <c r="X16" s="2"/>
-      <c r="Y16" s="5"/>
-      <c r="Z16" s="46"/>
-      <c r="AA16" s="5"/>
-      <c r="AB16" s="18"/>
-    </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C16" s="1"/>
+      <c r="D16" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" t="s">
+        <v>37</v>
+      </c>
+      <c r="I16" s="44"/>
+      <c r="J16" s="45"/>
+      <c r="K16" s="46"/>
+      <c r="L16" s="45"/>
+      <c r="M16" s="46"/>
+      <c r="N16" s="45"/>
+      <c r="O16" s="47"/>
+      <c r="Q16" s="16"/>
+      <c r="R16" s="6"/>
+      <c r="S16" s="3"/>
+      <c r="T16" s="41"/>
+      <c r="U16" s="3"/>
+      <c r="V16" s="6"/>
+      <c r="W16" s="19"/>
+      <c r="Y16" s="105"/>
+      <c r="Z16" s="5"/>
+      <c r="AA16" s="2"/>
+      <c r="AB16" s="5"/>
+      <c r="AC16" s="46"/>
+      <c r="AD16" s="5"/>
+      <c r="AE16" s="18"/>
+    </row>
+    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="50"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="49"/>
-      <c r="I17" s="48"/>
-      <c r="J17" s="49"/>
-      <c r="K17" s="48"/>
-      <c r="L17" s="54"/>
-      <c r="N17" s="16"/>
-      <c r="O17" s="6"/>
-      <c r="P17" s="3"/>
-      <c r="Q17" s="41"/>
-      <c r="R17" s="3"/>
-      <c r="S17" s="6"/>
-      <c r="T17" s="19"/>
-      <c r="V17" s="106"/>
-      <c r="W17" s="7"/>
-      <c r="X17" s="4"/>
-      <c r="Y17" s="7"/>
-      <c r="Z17" s="49"/>
-      <c r="AA17" s="7"/>
-      <c r="AB17" s="15"/>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C17" s="1"/>
+      <c r="I17" s="50"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="49"/>
+      <c r="L17" s="48"/>
+      <c r="M17" s="49"/>
+      <c r="N17" s="48"/>
+      <c r="O17" s="54"/>
+      <c r="Q17" s="16"/>
+      <c r="R17" s="6"/>
+      <c r="S17" s="3"/>
+      <c r="T17" s="41"/>
+      <c r="U17" s="3"/>
+      <c r="V17" s="6"/>
+      <c r="W17" s="19"/>
+      <c r="Y17" s="106"/>
+      <c r="Z17" s="7"/>
+      <c r="AA17" s="4"/>
+      <c r="AB17" s="7"/>
+      <c r="AC17" s="49"/>
+      <c r="AD17" s="7"/>
+      <c r="AE17" s="15"/>
+    </row>
+    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F18" s="40"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="41"/>
-      <c r="J18" s="42"/>
-      <c r="K18" s="41"/>
-      <c r="L18" s="43"/>
-      <c r="N18" s="44"/>
-      <c r="O18" s="5"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="5"/>
-      <c r="R18" s="113"/>
-      <c r="S18" s="5"/>
-      <c r="T18" s="18"/>
-      <c r="V18" s="16"/>
-      <c r="W18" s="41"/>
-      <c r="X18" s="3"/>
-      <c r="Y18" s="6"/>
-      <c r="Z18" s="3"/>
-      <c r="AA18" s="41"/>
-      <c r="AB18" s="19"/>
-    </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C18" s="1"/>
+      <c r="D18" t="s">
+        <v>36</v>
+      </c>
+      <c r="E18" t="s">
+        <v>35</v>
+      </c>
+      <c r="I18" s="40"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="42"/>
+      <c r="L18" s="41"/>
+      <c r="M18" s="42"/>
+      <c r="N18" s="41"/>
+      <c r="O18" s="43"/>
+      <c r="Q18" s="44"/>
+      <c r="R18" s="5"/>
+      <c r="S18" s="2"/>
+      <c r="T18" s="5"/>
+      <c r="U18" s="113"/>
+      <c r="V18" s="5"/>
+      <c r="W18" s="18"/>
+      <c r="Y18" s="16"/>
+      <c r="Z18" s="41"/>
+      <c r="AA18" s="3"/>
+      <c r="AB18" s="6"/>
+      <c r="AC18" s="3"/>
+      <c r="AD18" s="41"/>
+      <c r="AE18" s="19"/>
+    </row>
+    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F19" s="40"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="41"/>
-      <c r="J19" s="42"/>
-      <c r="K19" s="41"/>
-      <c r="L19" s="43"/>
-      <c r="N19" s="50"/>
-      <c r="O19" s="7"/>
-      <c r="P19" s="4"/>
-      <c r="Q19" s="7"/>
-      <c r="R19" s="114"/>
-      <c r="S19" s="7"/>
-      <c r="T19" s="15"/>
-      <c r="V19" s="16"/>
-      <c r="W19" s="41"/>
-      <c r="X19" s="3"/>
-      <c r="Y19" s="6"/>
-      <c r="Z19" s="3"/>
-      <c r="AA19" s="64"/>
-      <c r="AB19" s="19"/>
-    </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C19" s="1"/>
+      <c r="I19" s="40"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="41"/>
+      <c r="M19" s="42"/>
+      <c r="N19" s="41"/>
+      <c r="O19" s="43"/>
+      <c r="Q19" s="50"/>
+      <c r="R19" s="7"/>
+      <c r="S19" s="4"/>
+      <c r="T19" s="7"/>
+      <c r="U19" s="110"/>
+      <c r="V19" s="7"/>
+      <c r="W19" s="15"/>
+      <c r="Y19" s="16"/>
+      <c r="Z19" s="41"/>
+      <c r="AA19" s="3"/>
+      <c r="AB19" s="6"/>
+      <c r="AC19" s="3"/>
+      <c r="AD19" s="64"/>
+      <c r="AE19" s="19"/>
+    </row>
+    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F20" s="44"/>
-      <c r="G20" s="45"/>
-      <c r="H20" s="46"/>
-      <c r="I20" s="45"/>
-      <c r="J20" s="46"/>
-      <c r="K20" s="45"/>
-      <c r="L20" s="47"/>
-      <c r="N20" s="16"/>
-      <c r="O20" s="104"/>
-      <c r="P20" s="3"/>
-      <c r="Q20" s="6"/>
-      <c r="R20" s="3"/>
-      <c r="S20" s="34"/>
-      <c r="T20" s="19"/>
-      <c r="V20" s="17"/>
-      <c r="W20" s="5"/>
-      <c r="X20" s="100"/>
-      <c r="Y20" s="5"/>
-      <c r="Z20" s="2"/>
-      <c r="AA20" s="5"/>
-      <c r="AB20" s="67"/>
-    </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C20" s="1"/>
+      <c r="D20" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20" t="s">
+        <v>35</v>
+      </c>
+      <c r="I20" s="44"/>
+      <c r="J20" s="45"/>
+      <c r="K20" s="46"/>
+      <c r="L20" s="45"/>
+      <c r="M20" s="46"/>
+      <c r="N20" s="45"/>
+      <c r="O20" s="47"/>
+      <c r="Q20" s="16"/>
+      <c r="R20" s="104"/>
+      <c r="S20" s="3"/>
+      <c r="T20" s="6"/>
+      <c r="U20" s="3"/>
+      <c r="V20" s="34"/>
+      <c r="W20" s="19"/>
+      <c r="Y20" s="17"/>
+      <c r="Z20" s="5"/>
+      <c r="AA20" s="100"/>
+      <c r="AB20" s="5"/>
+      <c r="AC20" s="2"/>
+      <c r="AD20" s="5"/>
+      <c r="AE20" s="67"/>
+    </row>
+    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F21" s="50"/>
-      <c r="G21" s="48"/>
-      <c r="H21" s="49"/>
-      <c r="I21" s="48"/>
-      <c r="J21" s="49"/>
-      <c r="K21" s="48"/>
-      <c r="L21" s="54"/>
-      <c r="N21" s="16"/>
-      <c r="O21" s="84"/>
-      <c r="P21" s="3"/>
-      <c r="Q21" s="6"/>
-      <c r="R21" s="3"/>
-      <c r="S21" s="96"/>
-      <c r="T21" s="19"/>
-      <c r="V21" s="14"/>
-      <c r="W21" s="7"/>
-      <c r="X21" s="101"/>
-      <c r="Y21" s="7"/>
-      <c r="Z21" s="4"/>
-      <c r="AA21" s="7"/>
-      <c r="AB21" s="102"/>
-    </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C21" s="1"/>
+      <c r="I21" s="50"/>
+      <c r="J21" s="48"/>
+      <c r="K21" s="49"/>
+      <c r="L21" s="48"/>
+      <c r="M21" s="49"/>
+      <c r="N21" s="48"/>
+      <c r="O21" s="54"/>
+      <c r="Q21" s="16"/>
+      <c r="R21" s="84"/>
+      <c r="S21" s="3"/>
+      <c r="T21" s="6"/>
+      <c r="U21" s="3"/>
+      <c r="V21" s="96"/>
+      <c r="W21" s="19"/>
+      <c r="Y21" s="14"/>
+      <c r="Z21" s="7"/>
+      <c r="AA21" s="101"/>
+      <c r="AB21" s="7"/>
+      <c r="AC21" s="4"/>
+      <c r="AD21" s="7"/>
+      <c r="AE21" s="102"/>
+    </row>
+    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F22" s="40"/>
-      <c r="G22" s="41"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="41"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="6"/>
-      <c r="L22" s="43"/>
-      <c r="N22" s="17"/>
-      <c r="O22" s="5"/>
-      <c r="P22" s="65"/>
-      <c r="Q22" s="5"/>
-      <c r="R22" s="2"/>
-      <c r="S22" s="5"/>
-      <c r="T22" s="115"/>
-      <c r="V22" s="24"/>
-      <c r="W22" s="8"/>
-      <c r="X22" s="9"/>
-      <c r="Y22" s="112"/>
-      <c r="Z22" s="3"/>
-      <c r="AA22" s="6"/>
-      <c r="AB22" s="19"/>
-    </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C22" s="1"/>
+      <c r="D22" t="s">
+        <v>35</v>
+      </c>
+      <c r="E22" t="s">
+        <v>36</v>
+      </c>
+      <c r="I22" s="40"/>
+      <c r="J22" s="41"/>
+      <c r="K22" s="42"/>
+      <c r="L22" s="41"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="6"/>
+      <c r="O22" s="43"/>
+      <c r="Q22" s="17"/>
+      <c r="R22" s="5"/>
+      <c r="S22" s="65"/>
+      <c r="T22" s="5"/>
+      <c r="U22" s="2"/>
+      <c r="V22" s="5"/>
+      <c r="W22" s="114"/>
+      <c r="Y22" s="24"/>
+      <c r="Z22" s="8"/>
+      <c r="AA22" s="9"/>
+      <c r="AB22" s="112"/>
+      <c r="AC22" s="3"/>
+      <c r="AD22" s="6"/>
+      <c r="AE22" s="19"/>
+    </row>
+    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F23" s="82"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="6"/>
-      <c r="L23" s="43"/>
-      <c r="N23" s="14"/>
-      <c r="O23" s="7"/>
-      <c r="P23" s="71"/>
-      <c r="Q23" s="7"/>
-      <c r="R23" s="4"/>
-      <c r="S23" s="7"/>
-      <c r="T23" s="111"/>
-      <c r="V23" s="24"/>
-      <c r="W23" s="8"/>
-      <c r="X23" s="9"/>
-      <c r="Y23" s="64"/>
-      <c r="Z23" s="3"/>
-      <c r="AA23" s="6"/>
-      <c r="AB23" s="19"/>
-    </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C23" s="1"/>
+      <c r="I23" s="82"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="6"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="43"/>
+      <c r="Q23" s="14"/>
+      <c r="R23" s="7"/>
+      <c r="S23" s="71"/>
+      <c r="T23" s="7"/>
+      <c r="U23" s="4"/>
+      <c r="V23" s="7"/>
+      <c r="W23" s="111"/>
+      <c r="Y23" s="24"/>
+      <c r="Z23" s="8"/>
+      <c r="AA23" s="9"/>
+      <c r="AB23" s="64"/>
+      <c r="AC23" s="3"/>
+      <c r="AD23" s="6"/>
+      <c r="AE23" s="19"/>
+    </row>
+    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F24" s="17"/>
-      <c r="G24" s="69"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="69"/>
-      <c r="L24" s="18"/>
-      <c r="N24" s="16"/>
-      <c r="O24" s="6"/>
-      <c r="P24" s="3"/>
-      <c r="Q24" s="64"/>
-      <c r="R24" s="3"/>
-      <c r="S24" s="6"/>
-      <c r="T24" s="19"/>
-      <c r="V24" s="99"/>
-      <c r="W24" s="10"/>
-      <c r="X24" s="11"/>
-      <c r="Y24" s="5"/>
-      <c r="Z24" s="100"/>
-      <c r="AA24" s="5"/>
-      <c r="AB24" s="18"/>
-    </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C24" s="1"/>
+      <c r="D24" t="s">
+        <v>35</v>
+      </c>
+      <c r="E24" t="s">
+        <v>37</v>
+      </c>
+      <c r="I24" s="17"/>
+      <c r="J24" s="69"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="2"/>
+      <c r="N24" s="69"/>
+      <c r="O24" s="18"/>
+      <c r="Q24" s="16"/>
+      <c r="R24" s="6"/>
+      <c r="S24" s="3"/>
+      <c r="T24" s="64"/>
+      <c r="U24" s="3"/>
+      <c r="V24" s="6"/>
+      <c r="W24" s="19"/>
+      <c r="Y24" s="99"/>
+      <c r="Z24" s="10"/>
+      <c r="AA24" s="11"/>
+      <c r="AB24" s="5"/>
+      <c r="AC24" s="100"/>
+      <c r="AD24" s="5"/>
+      <c r="AE24" s="18"/>
+    </row>
+    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F25" s="14"/>
-      <c r="G25" s="70"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="7"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="70"/>
-      <c r="L25" s="15"/>
-      <c r="N25" s="16"/>
-      <c r="O25" s="6"/>
-      <c r="P25" s="3"/>
-      <c r="Q25" s="96"/>
-      <c r="R25" s="3"/>
-      <c r="S25" s="6"/>
-      <c r="T25" s="19"/>
-      <c r="V25" s="98"/>
-      <c r="W25" s="12"/>
-      <c r="X25" s="13"/>
-      <c r="Y25" s="7"/>
-      <c r="Z25" s="101"/>
-      <c r="AA25" s="7"/>
-      <c r="AB25" s="15"/>
-    </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C25" s="1"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="70"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="7"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="70"/>
+      <c r="O25" s="15"/>
+      <c r="Q25" s="16"/>
+      <c r="R25" s="6"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="96"/>
+      <c r="U25" s="3"/>
+      <c r="V25" s="6"/>
+      <c r="W25" s="19"/>
+      <c r="Y25" s="98"/>
+      <c r="Z25" s="12"/>
+      <c r="AA25" s="13"/>
+      <c r="AB25" s="7"/>
+      <c r="AC25" s="101"/>
+      <c r="AD25" s="7"/>
+      <c r="AE25" s="15"/>
+    </row>
+    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F26" s="40"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="42"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="6"/>
-      <c r="L26" s="19"/>
-      <c r="N26" s="94"/>
-      <c r="O26" s="80"/>
-      <c r="P26" s="2"/>
-      <c r="Q26" s="5"/>
-      <c r="R26" s="30"/>
-      <c r="S26" s="5"/>
-      <c r="T26" s="18"/>
-      <c r="V26" s="24"/>
-      <c r="W26" s="64"/>
-      <c r="X26" s="9"/>
-      <c r="Y26" s="6"/>
-      <c r="Z26" s="3"/>
-      <c r="AA26" s="64"/>
-      <c r="AB26" s="19"/>
-    </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C26" s="1"/>
+      <c r="D26" t="s">
+        <v>36</v>
+      </c>
+      <c r="E26" t="s">
+        <v>37</v>
+      </c>
+      <c r="I26" s="40"/>
+      <c r="J26" s="6"/>
+      <c r="K26" s="42"/>
+      <c r="L26" s="6"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="6"/>
+      <c r="O26" s="19"/>
+      <c r="Q26" s="94"/>
+      <c r="R26" s="80"/>
+      <c r="S26" s="2"/>
+      <c r="T26" s="5"/>
+      <c r="U26" s="30"/>
+      <c r="V26" s="5"/>
+      <c r="W26" s="18"/>
+      <c r="Y26" s="24"/>
+      <c r="Z26" s="64"/>
+      <c r="AA26" s="9"/>
+      <c r="AB26" s="6"/>
+      <c r="AC26" s="3"/>
+      <c r="AD26" s="64"/>
+      <c r="AE26" s="19"/>
+    </row>
+    <row r="27" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F27" s="40"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="6"/>
-      <c r="J27" s="3"/>
-      <c r="K27" s="6"/>
-      <c r="L27" s="19"/>
-      <c r="N27" s="106"/>
-      <c r="O27" s="81"/>
-      <c r="P27" s="4"/>
-      <c r="Q27" s="7"/>
-      <c r="R27" s="31"/>
-      <c r="S27" s="7"/>
-      <c r="T27" s="15"/>
-      <c r="V27" s="24"/>
-      <c r="W27" s="96"/>
-      <c r="X27" s="9"/>
-      <c r="Y27" s="6"/>
-      <c r="Z27" s="3"/>
-      <c r="AA27" s="96"/>
-      <c r="AB27" s="19"/>
-    </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C27" s="1"/>
+      <c r="I27" s="40"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="6"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="19"/>
+      <c r="Q27" s="106"/>
+      <c r="R27" s="81"/>
+      <c r="S27" s="4"/>
+      <c r="T27" s="7"/>
+      <c r="U27" s="31"/>
+      <c r="V27" s="7"/>
+      <c r="W27" s="15"/>
+      <c r="Y27" s="24"/>
+      <c r="Z27" s="96"/>
+      <c r="AA27" s="9"/>
+      <c r="AB27" s="6"/>
+      <c r="AC27" s="3"/>
+      <c r="AD27" s="96"/>
+      <c r="AE27" s="19"/>
+    </row>
+    <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F28" s="44"/>
-      <c r="G28" s="45"/>
-      <c r="H28" s="46"/>
-      <c r="I28" s="45"/>
-      <c r="J28" s="46"/>
-      <c r="K28" s="45"/>
-      <c r="L28" s="47"/>
-      <c r="N28" s="16"/>
-      <c r="O28" s="112"/>
-      <c r="P28" s="3"/>
-      <c r="Q28" s="6"/>
-      <c r="R28" s="3"/>
-      <c r="S28" s="112"/>
-      <c r="T28" s="19"/>
-      <c r="V28" s="25"/>
-      <c r="W28" s="10"/>
-      <c r="X28" s="65"/>
-      <c r="Y28" s="5"/>
-      <c r="Z28" s="2"/>
-      <c r="AA28" s="5"/>
-      <c r="AB28" s="67"/>
-    </row>
-    <row r="29" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C28" s="1"/>
+      <c r="D28" t="s">
+        <v>37</v>
+      </c>
+      <c r="E28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I28" s="44"/>
+      <c r="J28" s="45"/>
+      <c r="K28" s="46"/>
+      <c r="L28" s="45"/>
+      <c r="M28" s="46"/>
+      <c r="N28" s="45"/>
+      <c r="O28" s="47"/>
+      <c r="Q28" s="16"/>
+      <c r="R28" s="112"/>
+      <c r="S28" s="3"/>
+      <c r="T28" s="6"/>
+      <c r="U28" s="3"/>
+      <c r="V28" s="112"/>
+      <c r="W28" s="19"/>
+      <c r="Y28" s="25"/>
+      <c r="Z28" s="10"/>
+      <c r="AA28" s="65"/>
+      <c r="AB28" s="5"/>
+      <c r="AC28" s="2"/>
+      <c r="AD28" s="5"/>
+      <c r="AE28" s="67"/>
+    </row>
+    <row r="29" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F29" s="20"/>
-      <c r="G29" s="51"/>
-      <c r="H29" s="52"/>
-      <c r="I29" s="51"/>
-      <c r="J29" s="52"/>
-      <c r="K29" s="51"/>
-      <c r="L29" s="53"/>
-      <c r="N29" s="20"/>
-      <c r="O29" s="95"/>
-      <c r="P29" s="28"/>
-      <c r="Q29" s="23"/>
-      <c r="R29" s="28"/>
-      <c r="S29" s="95"/>
-      <c r="T29" s="29"/>
-      <c r="V29" s="26"/>
-      <c r="W29" s="27"/>
-      <c r="X29" s="66"/>
-      <c r="Y29" s="23"/>
-      <c r="Z29" s="28"/>
-      <c r="AA29" s="23"/>
-      <c r="AB29" s="68"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C29" s="1"/>
+      <c r="I29" s="20"/>
+      <c r="J29" s="51"/>
+      <c r="K29" s="52"/>
+      <c r="L29" s="51"/>
+      <c r="M29" s="52"/>
+      <c r="N29" s="51"/>
+      <c r="O29" s="53"/>
+      <c r="Q29" s="20"/>
+      <c r="R29" s="95"/>
+      <c r="S29" s="28"/>
+      <c r="T29" s="23"/>
+      <c r="U29" s="28"/>
+      <c r="V29" s="95"/>
+      <c r="W29" s="29"/>
+      <c r="Y29" s="26"/>
+      <c r="Z29" s="27"/>
+      <c r="AA29" s="66"/>
+      <c r="AB29" s="23"/>
+      <c r="AC29" s="28"/>
+      <c r="AD29" s="23"/>
+      <c r="AE29" s="68"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="62"/>
       <c r="B34" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="33"/>
       <c r="B35" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="72"/>
       <c r="B37" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="32"/>
       <c r="B38" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="97"/>
       <c r="B40" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="79"/>
       <c r="B42" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="103"/>
       <c r="B43" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="83"/>
       <c r="B44" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="63"/>
       <c r="B46" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>22</v>
       </c>
-      <c r="D48" t="s">
+      <c r="G48" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="49" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D49" t="s">
+    <row r="49" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G49" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="50" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D50" t="s">
+    <row r="50" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G50" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="51" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D51" t="s">
+    <row r="51" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G51" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="52" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D52" t="s">
+    <row r="52" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G52" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="53" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G53" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1941,4 +2128,656 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B0D6E7A-7808-4311-964E-552052446565}">
+  <dimension ref="A1:Y48"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="9" max="10" width="30" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1">
+        <v>1</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2</v>
+      </c>
+      <c r="M1" s="1">
+        <v>3</v>
+      </c>
+      <c r="O1" s="1">
+        <v>4</v>
+      </c>
+      <c r="Q1" s="1">
+        <v>5</v>
+      </c>
+      <c r="S1" s="1">
+        <v>6</v>
+      </c>
+      <c r="U1" s="1">
+        <v>7</v>
+      </c>
+      <c r="W1" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="I2" s="119"/>
+      <c r="J2" s="119"/>
+      <c r="K2" s="119"/>
+      <c r="L2" s="119"/>
+      <c r="M2" s="119"/>
+      <c r="N2" s="119"/>
+      <c r="O2" s="119"/>
+      <c r="P2" s="119"/>
+      <c r="Q2" s="119"/>
+      <c r="R2" s="119"/>
+      <c r="S2" s="119"/>
+      <c r="T2" s="119"/>
+      <c r="U2" s="119"/>
+      <c r="V2" s="119"/>
+      <c r="W2" s="119"/>
+      <c r="X2" s="119"/>
+      <c r="Y2" s="119"/>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>1</v>
+      </c>
+      <c r="I3" s="119">
+        <v>0</v>
+      </c>
+      <c r="J3" s="119"/>
+      <c r="K3" s="119">
+        <v>1</v>
+      </c>
+      <c r="L3" s="119"/>
+      <c r="M3" s="119">
+        <v>0.1</v>
+      </c>
+      <c r="N3" s="119"/>
+      <c r="O3" s="119">
+        <v>2</v>
+      </c>
+      <c r="P3" s="119"/>
+      <c r="Q3" s="119">
+        <v>3</v>
+      </c>
+      <c r="R3" s="119"/>
+      <c r="S3" s="119">
+        <v>4</v>
+      </c>
+      <c r="T3" s="119"/>
+      <c r="U3" s="119">
+        <v>5</v>
+      </c>
+      <c r="V3" s="119"/>
+      <c r="W3" s="119" t="s">
+        <v>39</v>
+      </c>
+      <c r="X3" s="119"/>
+      <c r="Y3" s="119"/>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I4" s="119">
+        <v>0</v>
+      </c>
+      <c r="J4" s="119"/>
+      <c r="K4" s="119">
+        <v>0</v>
+      </c>
+      <c r="L4" s="119"/>
+      <c r="M4" s="119">
+        <v>0</v>
+      </c>
+      <c r="N4" s="119"/>
+      <c r="O4" s="119">
+        <v>0</v>
+      </c>
+      <c r="P4" s="119"/>
+      <c r="Q4" s="119">
+        <v>0</v>
+      </c>
+      <c r="R4" s="119"/>
+      <c r="S4" s="119">
+        <v>0</v>
+      </c>
+      <c r="T4" s="119"/>
+      <c r="U4" s="119">
+        <v>0</v>
+      </c>
+      <c r="V4" s="119"/>
+      <c r="W4" s="119">
+        <v>0</v>
+      </c>
+      <c r="X4" s="119"/>
+      <c r="Y4" s="119"/>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="I5" s="119"/>
+      <c r="J5" s="120"/>
+      <c r="K5" s="119"/>
+      <c r="L5" s="119"/>
+      <c r="M5" s="119"/>
+      <c r="N5" s="119"/>
+      <c r="O5" s="119"/>
+      <c r="P5" s="119"/>
+      <c r="Q5" s="119"/>
+      <c r="R5" s="119"/>
+      <c r="S5" s="119"/>
+      <c r="T5" s="119"/>
+      <c r="U5" s="119"/>
+      <c r="V5" s="119"/>
+      <c r="W5" s="119"/>
+      <c r="X5" s="119"/>
+      <c r="Y5" s="119"/>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" s="121">
+        <v>0</v>
+      </c>
+      <c r="J6" s="121">
+        <v>102.74</v>
+      </c>
+      <c r="K6" s="121">
+        <v>0</v>
+      </c>
+      <c r="L6" s="121">
+        <v>49.92</v>
+      </c>
+      <c r="M6" s="121">
+        <v>0</v>
+      </c>
+      <c r="N6" s="121"/>
+      <c r="O6" s="121">
+        <v>0</v>
+      </c>
+      <c r="P6" s="121">
+        <v>0.61</v>
+      </c>
+      <c r="Q6" s="116">
+        <v>22571.79</v>
+      </c>
+      <c r="R6" s="116">
+        <v>22492.29</v>
+      </c>
+      <c r="S6" s="116">
+        <v>22571.79</v>
+      </c>
+      <c r="T6" s="116">
+        <v>22492.29</v>
+      </c>
+      <c r="U6" s="121">
+        <v>0</v>
+      </c>
+      <c r="V6" s="121">
+        <v>2.33</v>
+      </c>
+      <c r="W6" s="121">
+        <v>0</v>
+      </c>
+      <c r="X6" s="122">
+        <v>0.61</v>
+      </c>
+      <c r="Y6" s="119"/>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I7" s="121">
+        <v>0</v>
+      </c>
+      <c r="J7" s="123"/>
+      <c r="K7" s="121">
+        <v>0</v>
+      </c>
+      <c r="L7" s="119"/>
+      <c r="M7" s="119"/>
+      <c r="N7" s="119"/>
+      <c r="O7" s="119"/>
+      <c r="P7" s="119"/>
+      <c r="Q7" s="119"/>
+      <c r="R7" s="119"/>
+      <c r="S7" s="119"/>
+      <c r="T7" s="119"/>
+      <c r="U7" s="119"/>
+      <c r="V7" s="119"/>
+      <c r="W7" s="119"/>
+      <c r="X7" s="119"/>
+      <c r="Y7" s="119"/>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" t="s">
+        <v>44</v>
+      </c>
+      <c r="I8" s="122"/>
+      <c r="J8" s="123"/>
+      <c r="K8" s="119"/>
+      <c r="L8" s="119"/>
+      <c r="M8" s="119"/>
+      <c r="N8" s="119"/>
+      <c r="O8" s="119"/>
+      <c r="P8" s="119"/>
+      <c r="Q8" s="119"/>
+      <c r="R8" s="119"/>
+      <c r="S8" s="119"/>
+      <c r="T8" s="119"/>
+      <c r="U8" s="119"/>
+      <c r="V8" s="119"/>
+      <c r="W8" s="119"/>
+      <c r="X8" s="119"/>
+      <c r="Y8" s="119"/>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" t="s">
+        <v>43</v>
+      </c>
+      <c r="I9" s="124"/>
+      <c r="J9" s="123"/>
+      <c r="K9" s="119"/>
+      <c r="L9" s="119"/>
+      <c r="M9" s="119"/>
+      <c r="N9" s="119"/>
+      <c r="O9" s="119"/>
+      <c r="P9" s="119"/>
+      <c r="Q9" s="119"/>
+      <c r="R9" s="119"/>
+      <c r="S9" s="119"/>
+      <c r="T9" s="119"/>
+      <c r="U9" s="119"/>
+      <c r="V9" s="119"/>
+      <c r="W9" s="119"/>
+      <c r="X9" s="119"/>
+      <c r="Y9" s="119"/>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" t="s">
+        <v>44</v>
+      </c>
+      <c r="I10" s="122"/>
+      <c r="J10" s="123"/>
+      <c r="K10" s="119"/>
+      <c r="L10" s="119"/>
+      <c r="M10" s="119"/>
+      <c r="N10" s="119"/>
+      <c r="O10" s="119"/>
+      <c r="P10" s="119"/>
+      <c r="Q10" s="119"/>
+      <c r="R10" s="119"/>
+      <c r="S10" s="119"/>
+      <c r="T10" s="119"/>
+      <c r="U10" s="119"/>
+      <c r="V10" s="119"/>
+      <c r="W10" s="119"/>
+      <c r="X10" s="119"/>
+      <c r="Y10" s="119"/>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="I11" s="124"/>
+      <c r="J11" s="123"/>
+      <c r="K11" s="119"/>
+      <c r="L11" s="119"/>
+      <c r="M11" s="119"/>
+      <c r="N11" s="119"/>
+      <c r="O11" s="119"/>
+      <c r="P11" s="119"/>
+      <c r="Q11" s="119"/>
+      <c r="R11" s="119"/>
+      <c r="S11" s="119"/>
+      <c r="T11" s="119"/>
+      <c r="U11" s="119"/>
+      <c r="V11" s="119"/>
+      <c r="W11" s="119"/>
+      <c r="X11" s="119"/>
+      <c r="Y11" s="119"/>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="I12" s="125"/>
+      <c r="J12" s="123"/>
+      <c r="K12" s="119"/>
+      <c r="L12" s="119"/>
+      <c r="M12" s="119"/>
+      <c r="N12" s="119"/>
+      <c r="O12" s="119"/>
+      <c r="P12" s="119"/>
+      <c r="Q12" s="119"/>
+      <c r="R12" s="119"/>
+      <c r="S12" s="119"/>
+      <c r="T12" s="119"/>
+      <c r="U12" s="119"/>
+      <c r="V12" s="119"/>
+      <c r="W12" s="119"/>
+      <c r="X12" s="119"/>
+      <c r="Y12" s="119"/>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="I13" s="125"/>
+      <c r="J13" s="123"/>
+      <c r="K13" s="119"/>
+      <c r="L13" s="119"/>
+      <c r="M13" s="119"/>
+      <c r="N13" s="119"/>
+      <c r="O13" s="119"/>
+      <c r="P13" s="119"/>
+      <c r="Q13" s="119"/>
+      <c r="R13" s="119"/>
+      <c r="S13" s="119"/>
+      <c r="T13" s="119"/>
+      <c r="U13" s="119"/>
+      <c r="V13" s="119"/>
+      <c r="W13" s="119"/>
+      <c r="X13" s="119"/>
+      <c r="Y13" s="119"/>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="I14" s="117"/>
+      <c r="J14" s="118"/>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="I15" s="117"/>
+      <c r="J15" s="118"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C27" s="1"/>
+      <c r="D27" t="s">
+        <v>35</v>
+      </c>
+      <c r="E27" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" s="1"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C29" s="1"/>
+      <c r="D29" t="s">
+        <v>36</v>
+      </c>
+      <c r="E29" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="1"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C31" s="1"/>
+      <c r="D31" t="s">
+        <v>37</v>
+      </c>
+      <c r="E31" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" s="1"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33" s="1"/>
+      <c r="D33" t="s">
+        <v>34</v>
+      </c>
+      <c r="E33" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" s="1"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C35" s="1"/>
+      <c r="D35" t="s">
+        <v>34</v>
+      </c>
+      <c r="E35" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="1"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37" s="1"/>
+      <c r="D37" t="s">
+        <v>36</v>
+      </c>
+      <c r="E37" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="1"/>
+      <c r="B38" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" s="1"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C39" s="1"/>
+      <c r="D39" t="s">
+        <v>37</v>
+      </c>
+      <c r="E39" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="1"/>
+      <c r="B40" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C40" s="1"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C41" s="1"/>
+      <c r="D41" t="s">
+        <v>35</v>
+      </c>
+      <c r="E41" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="1"/>
+      <c r="B42" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C42" s="1"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C43" s="1"/>
+      <c r="D43" t="s">
+        <v>35</v>
+      </c>
+      <c r="E43" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="1"/>
+      <c r="B44" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C44" s="1"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C45" s="1"/>
+      <c r="D45" t="s">
+        <v>36</v>
+      </c>
+      <c r="E45" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="1"/>
+      <c r="B46" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C46" s="1"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C47" s="1"/>
+      <c r="D47" t="s">
+        <v>37</v>
+      </c>
+      <c r="E47" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="1"/>
+      <c r="B48" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C48" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
low high investigation of cost weights
</commit_message>
<xml_diff>
--- a/aln_control/testCases.xlsx
+++ b/aln_control/testCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Promotion\neurolib\aln_control\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE2DE18-4A97-4965-A1F4-96147AF23582}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{168E638E-8C6C-4ECB-A6A2-D9CB0197281E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-3120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="60">
   <si>
     <t>TC</t>
   </si>
@@ -169,12 +169,60 @@
   </si>
   <si>
     <t>zero</t>
+  </si>
+  <si>
+    <t>different solutions with similar cost</t>
+  </si>
+  <si>
+    <t>same as 2</t>
+  </si>
+  <si>
+    <t>different pulse height according to inital condition</t>
+  </si>
+  <si>
+    <t>same small peak remains</t>
+  </si>
+  <si>
+    <t>same as 4</t>
+  </si>
+  <si>
+    <t>zero a : slow convergence or high frequency rate input for "None" descent</t>
+  </si>
+  <si>
+    <t>no change from initial random guess, zero initial condition yields small peak similar to 5b</t>
+  </si>
+  <si>
+    <t>no change from initial random guess, zero initial condition yields small peak similar to 6b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">random initial conditions not removed </t>
+  </si>
+  <si>
+    <t>zero: does not reach "good" result (as relict of zero gradients?), HS descent performs reasonably well with high frequency rate input</t>
+  </si>
+  <si>
+    <t>precision only</t>
+  </si>
+  <si>
+    <t>precision + energy just below maximum</t>
+  </si>
+  <si>
+    <t>precision + sparsity just below maximum</t>
+  </si>
+  <si>
+    <t>precision + energy just beyond zero control for one/ both inputs</t>
+  </si>
+  <si>
+    <t>precision + sparsity just beyond zero control for one/ both inputs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="169" formatCode="0.000"/>
+  </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -232,7 +280,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -308,6 +356,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="27">
     <border>
@@ -618,7 +672,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="126">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -735,21 +789,12 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="11" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -758,6 +803,30 @@
     </xf>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="169" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="169" fontId="6" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="169" fontId="7" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2132,15 +2201,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B0D6E7A-7808-4311-964E-552052446565}">
-  <dimension ref="A1:Y48"/>
+  <dimension ref="A1:Z48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="9" max="10" width="30" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="8" width="8.7109375" customWidth="1"/>
+    <col min="9" max="24" width="19.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>33</v>
@@ -2184,121 +2252,121 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="I2" s="119"/>
-      <c r="J2" s="119"/>
-      <c r="K2" s="119"/>
-      <c r="L2" s="119"/>
-      <c r="M2" s="119"/>
-      <c r="N2" s="119"/>
-      <c r="O2" s="119"/>
-      <c r="P2" s="119"/>
-      <c r="Q2" s="119"/>
-      <c r="R2" s="119"/>
-      <c r="S2" s="119"/>
-      <c r="T2" s="119"/>
-      <c r="U2" s="119"/>
-      <c r="V2" s="119"/>
-      <c r="W2" s="119"/>
-      <c r="X2" s="119"/>
-      <c r="Y2" s="119"/>
-    </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="I2" s="118"/>
+      <c r="J2" s="118"/>
+      <c r="K2" s="118"/>
+      <c r="L2" s="118"/>
+      <c r="M2" s="118"/>
+      <c r="N2" s="118"/>
+      <c r="O2" s="118"/>
+      <c r="P2" s="118"/>
+      <c r="Q2" s="118"/>
+      <c r="R2" s="118"/>
+      <c r="S2" s="118"/>
+      <c r="T2" s="118"/>
+      <c r="U2" s="118"/>
+      <c r="V2" s="118"/>
+      <c r="W2" s="118"/>
+      <c r="X2" s="118"/>
+      <c r="Y2" s="118"/>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="G3" t="s">
         <v>1</v>
       </c>
-      <c r="I3" s="119">
+      <c r="I3" s="118">
         <v>0</v>
       </c>
-      <c r="J3" s="119"/>
-      <c r="K3" s="119">
+      <c r="J3" s="118"/>
+      <c r="K3" s="118">
         <v>1</v>
       </c>
-      <c r="L3" s="119"/>
-      <c r="M3" s="119">
+      <c r="L3" s="118"/>
+      <c r="M3" s="118">
         <v>0.1</v>
       </c>
-      <c r="N3" s="119"/>
-      <c r="O3" s="119">
+      <c r="N3" s="118"/>
+      <c r="O3" s="118">
         <v>2</v>
       </c>
-      <c r="P3" s="119"/>
-      <c r="Q3" s="119">
+      <c r="P3" s="118"/>
+      <c r="Q3" s="118">
         <v>3</v>
       </c>
-      <c r="R3" s="119"/>
-      <c r="S3" s="119">
+      <c r="R3" s="118"/>
+      <c r="S3" s="118">
         <v>4</v>
       </c>
-      <c r="T3" s="119"/>
-      <c r="U3" s="119">
+      <c r="T3" s="118"/>
+      <c r="U3" s="118">
         <v>5</v>
       </c>
-      <c r="V3" s="119"/>
-      <c r="W3" s="119" t="s">
+      <c r="V3" s="118"/>
+      <c r="W3" s="118" t="s">
         <v>39</v>
       </c>
-      <c r="X3" s="119"/>
-      <c r="Y3" s="119"/>
-    </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="X3" s="118"/>
+      <c r="Y3" s="118"/>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="G4" t="s">
         <v>2</v>
       </c>
-      <c r="I4" s="119">
+      <c r="I4" s="118">
         <v>0</v>
       </c>
-      <c r="J4" s="119"/>
-      <c r="K4" s="119">
+      <c r="J4" s="118"/>
+      <c r="K4" s="118">
         <v>0</v>
       </c>
-      <c r="L4" s="119"/>
-      <c r="M4" s="119">
+      <c r="L4" s="118"/>
+      <c r="M4" s="118">
         <v>0</v>
       </c>
-      <c r="N4" s="119"/>
-      <c r="O4" s="119">
+      <c r="N4" s="118"/>
+      <c r="O4" s="118">
         <v>0</v>
       </c>
-      <c r="P4" s="119"/>
-      <c r="Q4" s="119">
+      <c r="P4" s="118"/>
+      <c r="Q4" s="118">
         <v>0</v>
       </c>
-      <c r="R4" s="119"/>
-      <c r="S4" s="119">
+      <c r="R4" s="118"/>
+      <c r="S4" s="118">
         <v>0</v>
       </c>
-      <c r="T4" s="119"/>
-      <c r="U4" s="119">
+      <c r="T4" s="118"/>
+      <c r="U4" s="118">
         <v>0</v>
       </c>
-      <c r="V4" s="119"/>
-      <c r="W4" s="119">
+      <c r="V4" s="118"/>
+      <c r="W4" s="118">
         <v>0</v>
       </c>
-      <c r="X4" s="119"/>
-      <c r="Y4" s="119"/>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="I5" s="119"/>
-      <c r="J5" s="120"/>
-      <c r="K5" s="119"/>
+      <c r="X4" s="118"/>
+      <c r="Y4" s="118"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="I5" s="118"/>
+      <c r="J5" s="119"/>
+      <c r="K5" s="118"/>
       <c r="L5" s="119"/>
-      <c r="M5" s="119"/>
-      <c r="N5" s="119"/>
-      <c r="O5" s="119"/>
-      <c r="P5" s="119"/>
-      <c r="Q5" s="119"/>
-      <c r="R5" s="119"/>
-      <c r="S5" s="119"/>
-      <c r="T5" s="119"/>
-      <c r="U5" s="119"/>
-      <c r="V5" s="119"/>
-      <c r="W5" s="119"/>
-      <c r="X5" s="119"/>
-      <c r="Y5" s="119"/>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="M5" s="118"/>
+      <c r="N5" s="118"/>
+      <c r="O5" s="118"/>
+      <c r="P5" s="118"/>
+      <c r="Q5" s="118"/>
+      <c r="R5" s="118"/>
+      <c r="S5" s="118"/>
+      <c r="T5" s="118"/>
+      <c r="U5" s="118"/>
+      <c r="V5" s="118"/>
+      <c r="W5" s="118"/>
+      <c r="X5" s="118"/>
+      <c r="Y5" s="118"/>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -2308,61 +2376,63 @@
       <c r="C6" t="s">
         <v>35</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="I6" s="121">
+      <c r="I6" s="125">
         <v>0</v>
       </c>
-      <c r="J6" s="121">
-        <v>102.74</v>
-      </c>
-      <c r="K6" s="121">
+      <c r="J6" s="126">
+        <v>100.568</v>
+      </c>
+      <c r="K6" s="127">
         <v>0</v>
       </c>
-      <c r="L6" s="121">
-        <v>49.92</v>
-      </c>
-      <c r="M6" s="121">
+      <c r="L6" s="126">
+        <v>49.25</v>
+      </c>
+      <c r="M6" s="127">
         <v>0</v>
       </c>
-      <c r="N6" s="121"/>
-      <c r="O6" s="121">
+      <c r="N6" s="127">
+        <v>49.371000000000002</v>
+      </c>
+      <c r="O6" s="127">
         <v>0</v>
       </c>
-      <c r="P6" s="121">
+      <c r="P6" s="130">
         <v>0.61</v>
       </c>
-      <c r="Q6" s="116">
-        <v>22571.79</v>
-      </c>
-      <c r="R6" s="116">
-        <v>22492.29</v>
-      </c>
-      <c r="S6" s="116">
-        <v>22571.79</v>
-      </c>
-      <c r="T6" s="116">
-        <v>22492.29</v>
-      </c>
-      <c r="U6" s="121">
+      <c r="Q6" s="131">
+        <v>22571.788</v>
+      </c>
+      <c r="R6" s="132">
+        <v>22492.291000000001</v>
+      </c>
+      <c r="S6" s="132">
+        <v>22571.788</v>
+      </c>
+      <c r="T6" s="132">
+        <v>22492.177</v>
+      </c>
+      <c r="U6" s="133">
         <v>0</v>
       </c>
-      <c r="V6" s="121">
-        <v>2.33</v>
-      </c>
-      <c r="W6" s="121">
+      <c r="V6" s="133">
+        <v>2.327</v>
+      </c>
+      <c r="W6" s="133">
         <v>0</v>
       </c>
-      <c r="X6" s="122">
+      <c r="X6" s="133">
         <v>0.61</v>
       </c>
-      <c r="Y6" s="119"/>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y6" s="118"/>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -2372,169 +2442,331 @@
       <c r="E7" t="s">
         <v>42</v>
       </c>
-      <c r="I7" s="121">
-        <v>0</v>
-      </c>
-      <c r="J7" s="123"/>
-      <c r="K7" s="121">
-        <v>0</v>
-      </c>
-      <c r="L7" s="119"/>
-      <c r="M7" s="119"/>
-      <c r="N7" s="119"/>
-      <c r="O7" s="119"/>
-      <c r="P7" s="119"/>
-      <c r="Q7" s="119"/>
-      <c r="R7" s="119"/>
-      <c r="S7" s="119"/>
-      <c r="T7" s="119"/>
-      <c r="U7" s="119"/>
-      <c r="V7" s="119"/>
-      <c r="W7" s="119"/>
-      <c r="X7" s="119"/>
-      <c r="Y7" s="119"/>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="I7" s="123"/>
+      <c r="J7" s="127">
+        <v>100.566</v>
+      </c>
+      <c r="K7" s="123"/>
+      <c r="L7" s="126">
+        <v>49.354999999999997</v>
+      </c>
+      <c r="M7" s="123"/>
+      <c r="N7" s="127">
+        <v>49.368000000000002</v>
+      </c>
+      <c r="O7" s="123"/>
+      <c r="P7" s="129">
+        <v>0.61</v>
+      </c>
+      <c r="Q7" s="123"/>
+      <c r="R7" s="132">
+        <v>22492.291000000001</v>
+      </c>
+      <c r="S7" s="123"/>
+      <c r="T7" s="132">
+        <v>22492.177</v>
+      </c>
+      <c r="U7" s="123"/>
+      <c r="V7" s="133">
+        <v>2.327</v>
+      </c>
+      <c r="W7" s="123"/>
+      <c r="X7" s="133">
+        <v>0.61</v>
+      </c>
+      <c r="Y7" s="118"/>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
         <v>42</v>
       </c>
       <c r="E8" t="s">
         <v>44</v>
       </c>
-      <c r="I8" s="122"/>
-      <c r="J8" s="123"/>
-      <c r="K8" s="119"/>
-      <c r="L8" s="119"/>
-      <c r="M8" s="119"/>
-      <c r="N8" s="119"/>
-      <c r="O8" s="119"/>
-      <c r="P8" s="119"/>
-      <c r="Q8" s="119"/>
-      <c r="R8" s="119"/>
-      <c r="S8" s="119"/>
-      <c r="T8" s="119"/>
-      <c r="U8" s="119"/>
-      <c r="V8" s="119"/>
-      <c r="W8" s="119"/>
-      <c r="X8" s="119"/>
-      <c r="Y8" s="119"/>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="I8" s="123"/>
+      <c r="J8" s="127">
+        <v>100.566</v>
+      </c>
+      <c r="K8" s="123"/>
+      <c r="L8" s="126">
+        <v>49.354999999999997</v>
+      </c>
+      <c r="M8" s="123"/>
+      <c r="N8" s="129">
+        <v>49.36</v>
+      </c>
+      <c r="O8" s="123"/>
+      <c r="P8" s="129">
+        <v>0.61</v>
+      </c>
+      <c r="Q8" s="123"/>
+      <c r="R8" s="132">
+        <v>22492.291000000001</v>
+      </c>
+      <c r="S8" s="123"/>
+      <c r="T8" s="132">
+        <v>22492.177</v>
+      </c>
+      <c r="U8" s="123"/>
+      <c r="V8" s="133">
+        <v>2.327</v>
+      </c>
+      <c r="W8" s="123"/>
+      <c r="X8" s="129">
+        <v>0.61</v>
+      </c>
+      <c r="Y8" s="118"/>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
         <v>44</v>
       </c>
       <c r="E9" t="s">
         <v>43</v>
       </c>
-      <c r="I9" s="124"/>
-      <c r="J9" s="123"/>
-      <c r="K9" s="119"/>
-      <c r="L9" s="119"/>
-      <c r="M9" s="119"/>
-      <c r="N9" s="119"/>
-      <c r="O9" s="119"/>
-      <c r="P9" s="119"/>
-      <c r="Q9" s="119"/>
-      <c r="R9" s="119"/>
-      <c r="S9" s="119"/>
-      <c r="T9" s="119"/>
-      <c r="U9" s="119"/>
-      <c r="V9" s="119"/>
-      <c r="W9" s="119"/>
-      <c r="X9" s="119"/>
-      <c r="Y9" s="119"/>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="I9" s="127"/>
+      <c r="J9" s="127">
+        <v>100.568</v>
+      </c>
+      <c r="K9" s="124"/>
+      <c r="L9" s="126">
+        <v>49.25</v>
+      </c>
+      <c r="M9" s="124"/>
+      <c r="N9" s="124">
+        <v>49.366</v>
+      </c>
+      <c r="O9" s="124">
+        <v>0</v>
+      </c>
+      <c r="P9" s="129">
+        <v>0.61</v>
+      </c>
+      <c r="Q9" s="124">
+        <v>22492.031999999999</v>
+      </c>
+      <c r="R9" s="124">
+        <v>22492.287</v>
+      </c>
+      <c r="S9" s="124">
+        <v>22492.13</v>
+      </c>
+      <c r="T9" s="132">
+        <v>22492.173999999999</v>
+      </c>
+      <c r="U9" s="133">
+        <v>0</v>
+      </c>
+      <c r="V9" s="124">
+        <v>2.327</v>
+      </c>
+      <c r="W9" s="129">
+        <v>0</v>
+      </c>
+      <c r="X9" s="124">
+        <v>0.61</v>
+      </c>
+      <c r="Y9" s="118"/>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
         <v>44</v>
       </c>
       <c r="E10" t="s">
         <v>44</v>
       </c>
-      <c r="I10" s="122"/>
-      <c r="J10" s="123"/>
-      <c r="K10" s="119"/>
-      <c r="L10" s="119"/>
-      <c r="M10" s="119"/>
-      <c r="N10" s="119"/>
-      <c r="O10" s="119"/>
-      <c r="P10" s="119"/>
-      <c r="Q10" s="119"/>
-      <c r="R10" s="119"/>
-      <c r="S10" s="119"/>
-      <c r="T10" s="119"/>
-      <c r="U10" s="119"/>
-      <c r="V10" s="119"/>
-      <c r="W10" s="119"/>
-      <c r="X10" s="119"/>
-      <c r="Y10" s="119"/>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="I11" s="124"/>
-      <c r="J11" s="123"/>
-      <c r="K11" s="119"/>
-      <c r="L11" s="119"/>
-      <c r="M11" s="119"/>
-      <c r="N11" s="119"/>
-      <c r="O11" s="119"/>
-      <c r="P11" s="119"/>
-      <c r="Q11" s="119"/>
-      <c r="R11" s="119"/>
-      <c r="S11" s="119"/>
-      <c r="T11" s="119"/>
-      <c r="U11" s="119"/>
-      <c r="V11" s="119"/>
-      <c r="W11" s="119"/>
-      <c r="X11" s="119"/>
-      <c r="Y11" s="119"/>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="I12" s="125"/>
-      <c r="J12" s="123"/>
-      <c r="K12" s="119"/>
-      <c r="L12" s="119"/>
-      <c r="M12" s="119"/>
-      <c r="N12" s="119"/>
-      <c r="O12" s="119"/>
-      <c r="P12" s="119"/>
-      <c r="Q12" s="119"/>
-      <c r="R12" s="119"/>
-      <c r="S12" s="119"/>
-      <c r="T12" s="119"/>
-      <c r="U12" s="119"/>
-      <c r="V12" s="119"/>
-      <c r="W12" s="119"/>
-      <c r="X12" s="119"/>
-      <c r="Y12" s="119"/>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="I13" s="125"/>
-      <c r="J13" s="123"/>
-      <c r="K13" s="119"/>
-      <c r="L13" s="119"/>
-      <c r="M13" s="119"/>
-      <c r="N13" s="119"/>
-      <c r="O13" s="119"/>
-      <c r="P13" s="119"/>
-      <c r="Q13" s="119"/>
-      <c r="R13" s="119"/>
-      <c r="S13" s="119"/>
-      <c r="T13" s="119"/>
-      <c r="U13" s="119"/>
-      <c r="V13" s="119"/>
-      <c r="W13" s="119"/>
-      <c r="X13" s="119"/>
-      <c r="Y13" s="119"/>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="I14" s="117"/>
-      <c r="J14" s="118"/>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="I15" s="117"/>
-      <c r="J15" s="118"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I10" s="123"/>
+      <c r="J10" s="123">
+        <v>100.566</v>
+      </c>
+      <c r="K10" s="123"/>
+      <c r="L10" s="123"/>
+      <c r="M10" s="123"/>
+      <c r="N10" s="123"/>
+      <c r="O10" s="123"/>
+      <c r="P10" s="123"/>
+      <c r="Q10" s="123"/>
+      <c r="R10" s="123"/>
+      <c r="S10" s="123"/>
+      <c r="T10" s="123"/>
+      <c r="U10" s="123"/>
+      <c r="V10" s="123"/>
+      <c r="W10" s="123"/>
+      <c r="X10" s="123"/>
+      <c r="Y10" s="118"/>
+    </row>
+    <row r="11" spans="1:26" ht="90" x14ac:dyDescent="0.25">
+      <c r="I11" s="121"/>
+      <c r="J11" s="120"/>
+      <c r="K11" s="118"/>
+      <c r="L11" s="128" t="s">
+        <v>45</v>
+      </c>
+      <c r="M11" s="128"/>
+      <c r="N11" s="128" t="s">
+        <v>46</v>
+      </c>
+      <c r="O11" s="128" t="s">
+        <v>47</v>
+      </c>
+      <c r="P11" s="128"/>
+      <c r="Q11" s="128" t="s">
+        <v>51</v>
+      </c>
+      <c r="R11" s="128" t="s">
+        <v>48</v>
+      </c>
+      <c r="S11" s="128" t="s">
+        <v>52</v>
+      </c>
+      <c r="T11" s="128" t="s">
+        <v>48</v>
+      </c>
+      <c r="U11" s="128"/>
+      <c r="V11" s="128"/>
+      <c r="W11" s="128" t="s">
+        <v>53</v>
+      </c>
+      <c r="X11" s="128" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y11" s="118"/>
+    </row>
+    <row r="12" spans="1:26" ht="120" x14ac:dyDescent="0.25">
+      <c r="A12" s="134"/>
+      <c r="B12" s="134"/>
+      <c r="C12" s="134"/>
+      <c r="D12" s="134"/>
+      <c r="E12" s="134"/>
+      <c r="F12" s="134"/>
+      <c r="G12" s="134"/>
+      <c r="H12" s="134"/>
+      <c r="I12" s="135"/>
+      <c r="J12" s="136"/>
+      <c r="K12" s="128"/>
+      <c r="L12" s="128"/>
+      <c r="M12" s="128"/>
+      <c r="N12" s="128"/>
+      <c r="O12" s="128" t="s">
+        <v>50</v>
+      </c>
+      <c r="P12" s="128"/>
+      <c r="Q12" s="128"/>
+      <c r="R12" s="128"/>
+      <c r="S12" s="128"/>
+      <c r="T12" s="128"/>
+      <c r="U12" s="128" t="s">
+        <v>50</v>
+      </c>
+      <c r="V12" s="128"/>
+      <c r="W12" s="128" t="s">
+        <v>54</v>
+      </c>
+      <c r="X12" s="128"/>
+      <c r="Y12" s="128"/>
+      <c r="Z12" s="134"/>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="I13" s="122"/>
+      <c r="J13" s="120"/>
+      <c r="K13" s="118"/>
+      <c r="L13" s="128"/>
+      <c r="M13" s="128"/>
+      <c r="N13" s="128"/>
+      <c r="O13" s="128"/>
+      <c r="P13" s="128"/>
+      <c r="Q13" s="128"/>
+      <c r="R13" s="128"/>
+      <c r="S13" s="128"/>
+      <c r="T13" s="128"/>
+      <c r="U13" s="128"/>
+      <c r="V13" s="128"/>
+      <c r="W13" s="128"/>
+      <c r="X13" s="128"/>
+      <c r="Y13" s="118"/>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>55</v>
+      </c>
+      <c r="I14" s="116"/>
+      <c r="J14" s="117"/>
+      <c r="L14" s="134"/>
+      <c r="M14" s="134"/>
+      <c r="N14" s="134"/>
+      <c r="O14" s="134"/>
+      <c r="P14" s="134"/>
+      <c r="Q14" s="134"/>
+      <c r="R14" s="134"/>
+      <c r="S14" s="134"/>
+      <c r="T14" s="134"/>
+      <c r="U14" s="134"/>
+      <c r="V14" s="134"/>
+      <c r="W14" s="134"/>
+      <c r="X14" s="134"/>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
+        <v>56</v>
+      </c>
+      <c r="I15" s="116"/>
+      <c r="J15" s="117"/>
+      <c r="L15" s="134"/>
+      <c r="M15" s="134"/>
+      <c r="N15" s="134"/>
+      <c r="O15" s="134"/>
+      <c r="P15" s="134"/>
+      <c r="Q15" s="134"/>
+      <c r="R15" s="134"/>
+      <c r="S15" s="134"/>
+      <c r="T15" s="134"/>
+      <c r="U15" s="134"/>
+      <c r="V15" s="134"/>
+      <c r="W15" s="134"/>
+      <c r="X15" s="134"/>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L16" s="134"/>
+      <c r="M16" s="134"/>
+      <c r="N16" s="134"/>
+      <c r="O16" s="134"/>
+      <c r="P16" s="134"/>
+      <c r="Q16" s="134"/>
+      <c r="R16" s="134"/>
+      <c r="S16" s="134"/>
+      <c r="T16" s="134"/>
+      <c r="U16" s="134"/>
+      <c r="V16" s="134"/>
+      <c r="W16" s="134"/>
+      <c r="X16" s="134"/>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="D17" t="s">
+        <v>57</v>
+      </c>
+      <c r="L17" s="134"/>
+      <c r="M17" s="134"/>
+      <c r="N17" s="134"/>
+      <c r="O17" s="134"/>
+      <c r="P17" s="134"/>
+      <c r="Q17" s="134"/>
+      <c r="R17" s="134"/>
+      <c r="S17" s="134"/>
+      <c r="T17" s="134"/>
+      <c r="U17" s="134"/>
+      <c r="V17" s="134"/>
+      <c r="W17" s="134"/>
+      <c r="X17" s="134"/>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="D18" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>4</v>
       </c>
@@ -2549,14 +2781,14 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C28" s="1"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>5</v>
       </c>
@@ -2571,14 +2803,14 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C30" s="1"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>6</v>
       </c>
@@ -2593,7 +2825,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="1" t="s">
         <v>16</v>

</xml_diff>